<commit_message>
Added directionality to output. Added ability to define user clocks and gigabit tranceivers
</commit_message>
<xml_diff>
--- a/Verilog_Scripting/FMC_Definition_Template.xlsx
+++ b/Verilog_Scripting/FMC_Definition_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geesamen\Documents\GitProjects\EES_REPO_CTRL\Verilog_Scripting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3010F203-DF1A-45B7-8B53-5A4BE7E7E027}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{060E377B-ADAB-441E-A0A0-47E1DEC34EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41790" yWindow="2925" windowWidth="28800" windowHeight="15345" xr2:uid="{437B26FD-CA52-4A59-BAB8-AB7DC2C08C32}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{437B26FD-CA52-4A59-BAB8-AB7DC2C08C32}"/>
   </bookViews>
   <sheets>
     <sheet name="HPC_Setup_Sheet" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="239">
   <si>
     <t>CLK3_BIDIR_P</t>
   </si>
@@ -738,6 +738,24 @@
   </si>
   <si>
     <t>Output</t>
+  </si>
+  <si>
+    <t>Bob_P</t>
+  </si>
+  <si>
+    <t>Bob_N</t>
+  </si>
+  <si>
+    <t>Sally_P</t>
+  </si>
+  <si>
+    <t>Sally_N</t>
+  </si>
+  <si>
+    <t>James_P</t>
+  </si>
+  <si>
+    <t>James_N</t>
   </si>
 </sst>
 </file>
@@ -7193,6 +7211,9 @@
       <c r="B50" s="3" t="s">
         <v>144</v>
       </c>
+      <c r="C50" t="s">
+        <v>233</v>
+      </c>
       <c r="D50" t="s">
         <v>231</v>
       </c>
@@ -7204,6 +7225,9 @@
       <c r="B51" s="3" t="s">
         <v>145</v>
       </c>
+      <c r="C51" t="s">
+        <v>234</v>
+      </c>
       <c r="D51" t="s">
         <v>231</v>
       </c>
@@ -7369,6 +7393,9 @@
       <c r="B66" s="4" t="s">
         <v>160</v>
       </c>
+      <c r="C66" t="s">
+        <v>235</v>
+      </c>
       <c r="D66" t="s">
         <v>231</v>
       </c>
@@ -7380,6 +7407,9 @@
       <c r="B67" s="4" t="s">
         <v>161</v>
       </c>
+      <c r="C67" t="s">
+        <v>236</v>
+      </c>
       <c r="D67" t="s">
         <v>231</v>
       </c>
@@ -7391,6 +7421,9 @@
       <c r="B68" s="4" t="s">
         <v>162</v>
       </c>
+      <c r="C68" t="s">
+        <v>237</v>
+      </c>
       <c r="D68" t="s">
         <v>231</v>
       </c>
@@ -7401,6 +7434,9 @@
       </c>
       <c r="B69" s="4" t="s">
         <v>163</v>
+      </c>
+      <c r="C69" t="s">
+        <v>238</v>
       </c>
       <c r="D69" t="s">
         <v>231</v>
@@ -8230,9 +8266,9 @@
         <f>LPC_Setup_Sheet!B50</f>
         <v>GBTCLK0_M2C_P</v>
       </c>
-      <c r="B50">
+      <c r="B50" t="str">
         <f>LPC_Setup_Sheet!C50</f>
-        <v>0</v>
+        <v>Bob_P</v>
       </c>
       <c r="C50" t="str">
         <f>LPC_Setup_Sheet!D50</f>
@@ -8244,9 +8280,9 @@
         <f>LPC_Setup_Sheet!B51</f>
         <v>GBTCLK0_M2C_N</v>
       </c>
-      <c r="B51">
+      <c r="B51" t="str">
         <f>LPC_Setup_Sheet!C51</f>
-        <v>0</v>
+        <v>Bob_N</v>
       </c>
       <c r="C51" t="str">
         <f>LPC_Setup_Sheet!D51</f>
@@ -8454,9 +8490,9 @@
         <f>LPC_Setup_Sheet!B66</f>
         <v>DP0_C2M_P</v>
       </c>
-      <c r="B66">
+      <c r="B66" t="str">
         <f>LPC_Setup_Sheet!C66</f>
-        <v>0</v>
+        <v>Sally_P</v>
       </c>
       <c r="C66" t="str">
         <f>LPC_Setup_Sheet!D66</f>
@@ -8468,9 +8504,9 @@
         <f>LPC_Setup_Sheet!B67</f>
         <v>DP0_C2M_N</v>
       </c>
-      <c r="B67">
+      <c r="B67" t="str">
         <f>LPC_Setup_Sheet!C67</f>
-        <v>0</v>
+        <v>Sally_N</v>
       </c>
       <c r="C67" t="str">
         <f>LPC_Setup_Sheet!D67</f>
@@ -8482,9 +8518,9 @@
         <f>LPC_Setup_Sheet!B68</f>
         <v>DP0_M2C_P</v>
       </c>
-      <c r="B68">
+      <c r="B68" t="str">
         <f>LPC_Setup_Sheet!C68</f>
-        <v>0</v>
+        <v>James_P</v>
       </c>
       <c r="C68" t="str">
         <f>LPC_Setup_Sheet!D68</f>
@@ -8496,9 +8532,9 @@
         <f>LPC_Setup_Sheet!B69</f>
         <v>DP0_M2C_N</v>
       </c>
-      <c r="B69">
+      <c r="B69" t="str">
         <f>LPC_Setup_Sheet!C69</f>
-        <v>0</v>
+        <v>James_N</v>
       </c>
       <c r="C69" t="str">
         <f>LPC_Setup_Sheet!D69</f>

</xml_diff>

<commit_message>
Consolidated code and fixed issues with HPC definition and parsing.
</commit_message>
<xml_diff>
--- a/Verilog_Scripting/FMC_Definition_Template.xlsx
+++ b/Verilog_Scripting/FMC_Definition_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geesamen\Documents\GitProjects\EES_REPO_CTRL\Verilog_Scripting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{060E377B-ADAB-441E-A0A0-47E1DEC34EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1392C728-D988-47A2-ACFC-57CC6496E030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{437B26FD-CA52-4A59-BAB8-AB7DC2C08C32}"/>
+    <workbookView xWindow="-120" yWindow="0" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{437B26FD-CA52-4A59-BAB8-AB7DC2C08C32}"/>
   </bookViews>
   <sheets>
     <sheet name="HPC_Setup_Sheet" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="239">
   <si>
     <t>CLK3_BIDIR_P</t>
   </si>
@@ -1213,7 +1213,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D15412-8128-448E-B578-C5BF245D0FDB}">
-  <dimension ref="A1:W215"/>
+  <dimension ref="A1:W214"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.42578125" bestFit="1" customWidth="1"/>
@@ -1290,7 +1290,7 @@
         <v>216</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D6" t="s">
         <v>231</v>
@@ -1301,7 +1301,7 @@
         <v>216</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
         <v>231</v>
@@ -1312,7 +1312,7 @@
         <v>216</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D8" t="s">
         <v>231</v>
@@ -1323,7 +1323,7 @@
         <v>216</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
         <v>231</v>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
         <v>231</v>
@@ -1345,7 +1345,7 @@
         <v>220</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
         <v>231</v>
@@ -1353,10 +1353,10 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
         <v>231</v>
@@ -1367,7 +1367,7 @@
         <v>216</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
         <v>231</v>
@@ -1378,7 +1378,7 @@
         <v>216</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
         <v>231</v>
@@ -1389,7 +1389,7 @@
         <v>216</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D15" t="s">
         <v>231</v>
@@ -1397,10 +1397,10 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D16" t="s">
         <v>231</v>
@@ -1411,7 +1411,7 @@
         <v>220</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D17" t="s">
         <v>231</v>
@@ -1422,7 +1422,7 @@
         <v>220</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D18" t="s">
         <v>231</v>
@@ -1433,7 +1433,7 @@
         <v>220</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
         <v>231</v>
@@ -1441,10 +1441,10 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D20" t="s">
         <v>231</v>
@@ -1455,7 +1455,7 @@
         <v>216</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D21" t="s">
         <v>231</v>
@@ -1466,7 +1466,7 @@
         <v>216</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D22" t="s">
         <v>231</v>
@@ -1477,7 +1477,7 @@
         <v>216</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D23" t="s">
         <v>231</v>
@@ -1485,10 +1485,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
         <v>231</v>
@@ -1499,7 +1499,7 @@
         <v>220</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D25" t="s">
         <v>231</v>
@@ -1507,10 +1507,10 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>220</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>47</v>
+        <v>221</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="D26" t="s">
         <v>231</v>
@@ -1521,7 +1521,7 @@
         <v>221</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="s">
         <v>231</v>
@@ -1529,10 +1529,10 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>221</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>1</v>
+        <v>216</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="D28" t="s">
         <v>231</v>
@@ -1543,7 +1543,7 @@
         <v>216</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D29" t="s">
         <v>231</v>
@@ -1554,7 +1554,7 @@
         <v>216</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D30" t="s">
         <v>231</v>
@@ -1565,7 +1565,7 @@
         <v>216</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D31" t="s">
         <v>231</v>
@@ -1576,7 +1576,7 @@
         <v>216</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D32" t="s">
         <v>231</v>
@@ -1587,7 +1587,7 @@
         <v>216</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D33" t="s">
         <v>231</v>
@@ -1598,7 +1598,7 @@
         <v>216</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D34" t="s">
         <v>231</v>
@@ -1609,7 +1609,7 @@
         <v>216</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D35" t="s">
         <v>231</v>
@@ -1620,7 +1620,7 @@
         <v>216</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D36" t="s">
         <v>231</v>
@@ -1631,7 +1631,7 @@
         <v>216</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D37" t="s">
         <v>231</v>
@@ -1642,7 +1642,7 @@
         <v>216</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D38" t="s">
         <v>231</v>
@@ -1653,7 +1653,7 @@
         <v>216</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D39" t="s">
         <v>231</v>
@@ -1664,7 +1664,7 @@
         <v>216</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D40" t="s">
         <v>231</v>
@@ -1675,7 +1675,7 @@
         <v>216</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D41" t="s">
         <v>231</v>
@@ -1686,7 +1686,7 @@
         <v>216</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D42" t="s">
         <v>231</v>
@@ -1697,7 +1697,7 @@
         <v>216</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D43" t="s">
         <v>231</v>
@@ -1708,7 +1708,7 @@
         <v>216</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D44" t="s">
         <v>231</v>
@@ -1719,7 +1719,7 @@
         <v>216</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D45" t="s">
         <v>231</v>
@@ -1730,7 +1730,7 @@
         <v>216</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D46" t="s">
         <v>231</v>
@@ -1741,7 +1741,7 @@
         <v>216</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D47" t="s">
         <v>231</v>
@@ -1752,7 +1752,7 @@
         <v>216</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D48" t="s">
         <v>231</v>
@@ -1763,7 +1763,7 @@
         <v>216</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D49" t="s">
         <v>231</v>
@@ -1771,10 +1771,10 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>216</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>46</v>
+        <v>222</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="D50" t="s">
         <v>231</v>
@@ -1785,7 +1785,7 @@
         <v>222</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D51" t="s">
         <v>231</v>
@@ -1793,10 +1793,10 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>222</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>49</v>
+        <v>216</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="D52" t="s">
         <v>231</v>
@@ -1807,7 +1807,7 @@
         <v>216</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D53" t="s">
         <v>231</v>
@@ -1818,7 +1818,7 @@
         <v>216</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D54" t="s">
         <v>231</v>
@@ -1829,7 +1829,7 @@
         <v>216</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D55" t="s">
         <v>231</v>
@@ -1840,7 +1840,7 @@
         <v>216</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D56" t="s">
         <v>231</v>
@@ -1851,7 +1851,7 @@
         <v>216</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D57" t="s">
         <v>231</v>
@@ -1862,7 +1862,7 @@
         <v>216</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D58" t="s">
         <v>231</v>
@@ -1873,7 +1873,7 @@
         <v>216</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D59" t="s">
         <v>231</v>
@@ -1884,7 +1884,7 @@
         <v>216</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D60" t="s">
         <v>231</v>
@@ -1895,7 +1895,7 @@
         <v>216</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D61" t="s">
         <v>231</v>
@@ -1906,7 +1906,7 @@
         <v>216</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D62" t="s">
         <v>231</v>
@@ -1917,7 +1917,7 @@
         <v>216</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D63" t="s">
         <v>231</v>
@@ -1928,7 +1928,7 @@
         <v>216</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D64" t="s">
         <v>231</v>
@@ -1939,7 +1939,7 @@
         <v>216</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D65" t="s">
         <v>231</v>
@@ -1950,7 +1950,7 @@
         <v>216</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D66" t="s">
         <v>231</v>
@@ -1961,7 +1961,7 @@
         <v>216</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D67" t="s">
         <v>231</v>
@@ -1972,7 +1972,7 @@
         <v>216</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D68" t="s">
         <v>231</v>
@@ -1983,7 +1983,7 @@
         <v>216</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D69" t="s">
         <v>231</v>
@@ -1994,7 +1994,7 @@
         <v>216</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D70" t="s">
         <v>231</v>
@@ -2005,7 +2005,7 @@
         <v>216</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D71" t="s">
         <v>231</v>
@@ -2016,7 +2016,7 @@
         <v>216</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D72" t="s">
         <v>231</v>
@@ -2027,7 +2027,7 @@
         <v>216</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D73" t="s">
         <v>231</v>
@@ -2035,10 +2035,10 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>216</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>71</v>
+        <v>222</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="D74" t="s">
         <v>231</v>
@@ -2049,7 +2049,7 @@
         <v>222</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D75" t="s">
         <v>231</v>
@@ -2057,10 +2057,10 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>222</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>73</v>
+        <v>220</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>74</v>
       </c>
       <c r="D76" t="s">
         <v>231</v>
@@ -2071,7 +2071,7 @@
         <v>220</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D77" t="s">
         <v>231</v>
@@ -2079,10 +2079,10 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D78" t="s">
         <v>231</v>
@@ -2093,7 +2093,7 @@
         <v>216</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D79" t="s">
         <v>231</v>
@@ -2104,7 +2104,7 @@
         <v>216</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D80" t="s">
         <v>231</v>
@@ -2115,7 +2115,7 @@
         <v>216</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D81" t="s">
         <v>231</v>
@@ -2126,7 +2126,7 @@
         <v>216</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D82" t="s">
         <v>231</v>
@@ -2137,7 +2137,7 @@
         <v>216</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D83" t="s">
         <v>231</v>
@@ -2148,7 +2148,7 @@
         <v>216</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D84" t="s">
         <v>231</v>
@@ -2159,7 +2159,7 @@
         <v>216</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D85" t="s">
         <v>231</v>
@@ -2170,7 +2170,7 @@
         <v>216</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D86" t="s">
         <v>231</v>
@@ -2181,7 +2181,7 @@
         <v>216</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D87" t="s">
         <v>231</v>
@@ -2192,7 +2192,7 @@
         <v>216</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D88" t="s">
         <v>231</v>
@@ -2203,7 +2203,7 @@
         <v>216</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D89" t="s">
         <v>231</v>
@@ -2214,7 +2214,7 @@
         <v>216</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D90" t="s">
         <v>231</v>
@@ -2225,7 +2225,7 @@
         <v>216</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D91" t="s">
         <v>231</v>
@@ -2236,7 +2236,7 @@
         <v>216</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D92" t="s">
         <v>231</v>
@@ -2247,7 +2247,7 @@
         <v>216</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D93" t="s">
         <v>231</v>
@@ -2258,7 +2258,7 @@
         <v>216</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D94" t="s">
         <v>231</v>
@@ -2269,7 +2269,7 @@
         <v>216</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D95" t="s">
         <v>231</v>
@@ -2280,7 +2280,7 @@
         <v>216</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D96" t="s">
         <v>231</v>
@@ -2291,7 +2291,7 @@
         <v>216</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D97" t="s">
         <v>231</v>
@@ -2299,10 +2299,10 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D98" t="s">
         <v>231</v>
@@ -2313,7 +2313,7 @@
         <v>220</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D99" t="s">
         <v>231</v>
@@ -2321,10 +2321,10 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D100" t="s">
         <v>231</v>
@@ -2335,7 +2335,7 @@
         <v>216</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D101" t="s">
         <v>231</v>
@@ -2346,7 +2346,7 @@
         <v>216</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D102" t="s">
         <v>231</v>
@@ -2357,7 +2357,7 @@
         <v>216</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D103" t="s">
         <v>231</v>
@@ -2368,7 +2368,7 @@
         <v>216</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D104" t="s">
         <v>231</v>
@@ -2379,7 +2379,7 @@
         <v>216</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D105" t="s">
         <v>231</v>
@@ -2390,7 +2390,7 @@
         <v>216</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D106" t="s">
         <v>231</v>
@@ -2401,7 +2401,7 @@
         <v>216</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D107" t="s">
         <v>231</v>
@@ -2412,7 +2412,7 @@
         <v>216</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D108" t="s">
         <v>231</v>
@@ -2423,7 +2423,7 @@
         <v>216</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D109" t="s">
         <v>231</v>
@@ -2434,7 +2434,7 @@
         <v>216</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D110" t="s">
         <v>231</v>
@@ -2445,7 +2445,7 @@
         <v>216</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D111" t="s">
         <v>231</v>
@@ -2456,7 +2456,7 @@
         <v>216</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D112" t="s">
         <v>231</v>
@@ -2467,7 +2467,7 @@
         <v>216</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D113" t="s">
         <v>231</v>
@@ -2478,7 +2478,7 @@
         <v>216</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D114" t="s">
         <v>231</v>
@@ -2489,7 +2489,7 @@
         <v>216</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D115" t="s">
         <v>231</v>
@@ -2500,7 +2500,7 @@
         <v>216</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D116" t="s">
         <v>231</v>
@@ -2511,7 +2511,7 @@
         <v>216</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D117" t="s">
         <v>231</v>
@@ -2522,7 +2522,7 @@
         <v>216</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D118" t="s">
         <v>231</v>
@@ -2533,7 +2533,7 @@
         <v>216</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D119" t="s">
         <v>231</v>
@@ -2544,7 +2544,7 @@
         <v>216</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D120" t="s">
         <v>231</v>
@@ -2555,7 +2555,7 @@
         <v>216</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D121" t="s">
         <v>231</v>
@@ -2563,10 +2563,10 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D122" t="s">
         <v>231</v>
@@ -2577,7 +2577,7 @@
         <v>220</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D123" t="s">
         <v>231</v>
@@ -2585,10 +2585,10 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D124" t="s">
         <v>231</v>
@@ -2599,7 +2599,7 @@
         <v>216</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D125" t="s">
         <v>231</v>
@@ -2610,7 +2610,7 @@
         <v>216</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D126" t="s">
         <v>231</v>
@@ -2621,7 +2621,7 @@
         <v>216</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D127" t="s">
         <v>231</v>
@@ -2632,7 +2632,7 @@
         <v>216</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D128" t="s">
         <v>231</v>
@@ -2643,7 +2643,7 @@
         <v>216</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D129" t="s">
         <v>231</v>
@@ -2654,7 +2654,7 @@
         <v>216</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D130" t="s">
         <v>231</v>
@@ -2665,7 +2665,7 @@
         <v>216</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D131" t="s">
         <v>231</v>
@@ -2676,7 +2676,7 @@
         <v>216</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D132" t="s">
         <v>231</v>
@@ -2687,7 +2687,7 @@
         <v>216</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D133" t="s">
         <v>231</v>
@@ -2698,7 +2698,7 @@
         <v>216</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D134" t="s">
         <v>231</v>
@@ -2709,7 +2709,7 @@
         <v>216</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D135" t="s">
         <v>231</v>
@@ -2720,7 +2720,7 @@
         <v>216</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D136" t="s">
         <v>231</v>
@@ -2731,7 +2731,7 @@
         <v>216</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D137" t="s">
         <v>231</v>
@@ -2742,7 +2742,7 @@
         <v>216</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D138" t="s">
         <v>231</v>
@@ -2753,7 +2753,7 @@
         <v>216</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D139" t="s">
         <v>231</v>
@@ -2764,7 +2764,7 @@
         <v>216</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D140" t="s">
         <v>231</v>
@@ -2775,7 +2775,7 @@
         <v>216</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D141" t="s">
         <v>231</v>
@@ -2786,7 +2786,7 @@
         <v>216</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D142" t="s">
         <v>231</v>
@@ -2797,7 +2797,7 @@
         <v>216</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D143" t="s">
         <v>231</v>
@@ -2808,7 +2808,7 @@
         <v>216</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D144" t="s">
         <v>231</v>
@@ -2819,7 +2819,7 @@
         <v>216</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D145" t="s">
         <v>231</v>
@@ -2827,10 +2827,10 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>216</v>
-      </c>
-      <c r="B146" s="2" t="s">
-        <v>143</v>
+        <v>218</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>144</v>
       </c>
       <c r="D146" t="s">
         <v>231</v>
@@ -2841,7 +2841,7 @@
         <v>218</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D147" t="s">
         <v>231</v>
@@ -2849,10 +2849,10 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>218</v>
-      </c>
-      <c r="B148" s="3" t="s">
-        <v>145</v>
+        <v>220</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>146</v>
       </c>
       <c r="D148" t="s">
         <v>231</v>
@@ -2863,7 +2863,7 @@
         <v>220</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D149" t="s">
         <v>231</v>
@@ -2871,10 +2871,10 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D150" t="s">
         <v>231</v>
@@ -2885,7 +2885,7 @@
         <v>216</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D151" t="s">
         <v>231</v>
@@ -2896,7 +2896,7 @@
         <v>216</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D152" t="s">
         <v>231</v>
@@ -2907,7 +2907,7 @@
         <v>216</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D153" t="s">
         <v>231</v>
@@ -2918,7 +2918,7 @@
         <v>216</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D154" t="s">
         <v>231</v>
@@ -2929,7 +2929,7 @@
         <v>216</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D155" t="s">
         <v>231</v>
@@ -2937,10 +2937,10 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D156" t="s">
         <v>231</v>
@@ -2951,7 +2951,7 @@
         <v>220</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D157" t="s">
         <v>231</v>
@@ -2959,10 +2959,10 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D158" t="s">
         <v>231</v>
@@ -2973,7 +2973,7 @@
         <v>216</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D159" t="s">
         <v>231</v>
@@ -2984,7 +2984,7 @@
         <v>216</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D160" t="s">
         <v>231</v>
@@ -2995,7 +2995,7 @@
         <v>216</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D161" t="s">
         <v>231</v>
@@ -3003,10 +3003,10 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>216</v>
-      </c>
-      <c r="B162" s="2" t="s">
-        <v>159</v>
+        <v>217</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>160</v>
       </c>
       <c r="D162" t="s">
         <v>231</v>
@@ -3017,7 +3017,7 @@
         <v>217</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D163" t="s">
         <v>231</v>
@@ -3028,7 +3028,7 @@
         <v>217</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D164" t="s">
         <v>231</v>
@@ -3039,7 +3039,7 @@
         <v>217</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D165" t="s">
         <v>231</v>
@@ -3047,10 +3047,10 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>217</v>
-      </c>
-      <c r="B166" s="4" t="s">
-        <v>163</v>
+        <v>216</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>164</v>
       </c>
       <c r="D166" t="s">
         <v>231</v>
@@ -3061,7 +3061,7 @@
         <v>216</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D167" t="s">
         <v>231</v>
@@ -3072,7 +3072,7 @@
         <v>216</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D168" t="s">
         <v>231</v>
@@ -3083,7 +3083,7 @@
         <v>216</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D169" t="s">
         <v>231</v>
@@ -3094,7 +3094,7 @@
         <v>216</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D170" t="s">
         <v>231</v>
@@ -3105,7 +3105,7 @@
         <v>216</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D171" t="s">
         <v>231</v>
@@ -3113,10 +3113,10 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D172" t="s">
         <v>231</v>
@@ -3127,7 +3127,7 @@
         <v>220</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D173" t="s">
         <v>231</v>
@@ -3135,10 +3135,10 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D174" t="s">
         <v>231</v>
@@ -3149,7 +3149,7 @@
         <v>216</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D175" t="s">
         <v>231</v>
@@ -3157,10 +3157,10 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>216</v>
-      </c>
-      <c r="B176" s="2" t="s">
-        <v>173</v>
+        <v>219</v>
+      </c>
+      <c r="B176" s="1" t="s">
+        <v>174</v>
       </c>
       <c r="D176" t="s">
         <v>231</v>
@@ -3168,10 +3168,10 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>219</v>
-      </c>
-      <c r="B177" s="1" t="s">
-        <v>174</v>
+        <v>217</v>
+      </c>
+      <c r="B177" s="4" t="s">
+        <v>175</v>
       </c>
       <c r="D177" t="s">
         <v>231</v>
@@ -3182,7 +3182,7 @@
         <v>217</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D178" t="s">
         <v>231</v>
@@ -3193,7 +3193,7 @@
         <v>217</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D179" t="s">
         <v>231</v>
@@ -3204,7 +3204,7 @@
         <v>217</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D180" t="s">
         <v>231</v>
@@ -3215,7 +3215,7 @@
         <v>217</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D181" t="s">
         <v>231</v>
@@ -3226,7 +3226,7 @@
         <v>217</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D182" t="s">
         <v>231</v>
@@ -3237,7 +3237,7 @@
         <v>217</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D183" t="s">
         <v>231</v>
@@ -3248,7 +3248,7 @@
         <v>217</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D184" t="s">
         <v>231</v>
@@ -3256,10 +3256,10 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>217</v>
-      </c>
-      <c r="B185" s="4" t="s">
-        <v>182</v>
+        <v>218</v>
+      </c>
+      <c r="B185" s="3" t="s">
+        <v>183</v>
       </c>
       <c r="D185" t="s">
         <v>231</v>
@@ -3270,7 +3270,7 @@
         <v>218</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D186" t="s">
         <v>231</v>
@@ -3278,10 +3278,10 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>218</v>
-      </c>
-      <c r="B187" s="3" t="s">
-        <v>184</v>
+        <v>217</v>
+      </c>
+      <c r="B187" s="4" t="s">
+        <v>185</v>
       </c>
       <c r="D187" t="s">
         <v>231</v>
@@ -3292,7 +3292,7 @@
         <v>217</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D188" t="s">
         <v>231</v>
@@ -3303,7 +3303,7 @@
         <v>217</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D189" t="s">
         <v>231</v>
@@ -3314,7 +3314,7 @@
         <v>217</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D190" t="s">
         <v>231</v>
@@ -3325,7 +3325,7 @@
         <v>217</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D191" t="s">
         <v>231</v>
@@ -3336,7 +3336,7 @@
         <v>217</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D192" t="s">
         <v>231</v>
@@ -3347,7 +3347,7 @@
         <v>217</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D193" t="s">
         <v>231</v>
@@ -3358,7 +3358,7 @@
         <v>217</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D194" t="s">
         <v>231</v>
@@ -3369,7 +3369,7 @@
         <v>217</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D195" t="s">
         <v>231</v>
@@ -3380,7 +3380,7 @@
         <v>217</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D196" t="s">
         <v>231</v>
@@ -3391,7 +3391,7 @@
         <v>217</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D197" t="s">
         <v>231</v>
@@ -3402,7 +3402,7 @@
         <v>217</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D198" t="s">
         <v>231</v>
@@ -3413,7 +3413,7 @@
         <v>217</v>
       </c>
       <c r="B199" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D199" t="s">
         <v>231</v>
@@ -3424,7 +3424,7 @@
         <v>217</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D200" t="s">
         <v>231</v>
@@ -3435,7 +3435,7 @@
         <v>217</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D201" t="s">
         <v>231</v>
@@ -3446,7 +3446,7 @@
         <v>217</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D202" t="s">
         <v>231</v>
@@ -3457,7 +3457,7 @@
         <v>217</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D203" t="s">
         <v>231</v>
@@ -3468,7 +3468,7 @@
         <v>217</v>
       </c>
       <c r="B204" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D204" t="s">
         <v>231</v>
@@ -3479,7 +3479,7 @@
         <v>217</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D205" t="s">
         <v>231</v>
@@ -3490,7 +3490,7 @@
         <v>217</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D206" t="s">
         <v>231</v>
@@ -3501,7 +3501,7 @@
         <v>217</v>
       </c>
       <c r="B207" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D207" t="s">
         <v>231</v>
@@ -3512,7 +3512,7 @@
         <v>217</v>
       </c>
       <c r="B208" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D208" t="s">
         <v>231</v>
@@ -3523,7 +3523,7 @@
         <v>217</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D209" t="s">
         <v>231</v>
@@ -3534,7 +3534,7 @@
         <v>217</v>
       </c>
       <c r="B210" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D210" t="s">
         <v>231</v>
@@ -3545,7 +3545,7 @@
         <v>217</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D211" t="s">
         <v>231</v>
@@ -3556,7 +3556,7 @@
         <v>217</v>
       </c>
       <c r="B212" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D212" t="s">
         <v>231</v>
@@ -3567,7 +3567,7 @@
         <v>217</v>
       </c>
       <c r="B213" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D213" t="s">
         <v>231</v>
@@ -3578,25 +3578,14 @@
         <v>217</v>
       </c>
       <c r="B214" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D214" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A215" t="s">
-        <v>217</v>
-      </c>
-      <c r="B215" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="D215" t="s">
-        <v>231</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D215">
+  <conditionalFormatting sqref="D2:D214">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>$W$2</formula>
     </cfRule>
@@ -3605,7 +3594,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D215" xr:uid="{82DB2AE3-90C7-41CC-A067-2FC3C40EAA63}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D214" xr:uid="{82DB2AE3-90C7-41CC-A067-2FC3C40EAA63}">
       <formula1>$W$1:$W$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -3615,7 +3604,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CC6CFD7-6E6D-4D7E-A251-EBAA5E2EFA62}">
-  <dimension ref="A1:C215"/>
+  <dimension ref="A1:C214"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -3691,7 +3680,7 @@
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>HPC_Setup_Sheet!B6</f>
-        <v>HA02_N</v>
+        <v>HA06_P</v>
       </c>
       <c r="B6">
         <f>HPC_Setup_Sheet!C6</f>
@@ -3705,7 +3694,7 @@
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>HPC_Setup_Sheet!B7</f>
-        <v>HA06_P</v>
+        <v>HA06_N</v>
       </c>
       <c r="B7">
         <f>HPC_Setup_Sheet!C7</f>
@@ -3719,7 +3708,7 @@
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>HPC_Setup_Sheet!B8</f>
-        <v>HA06_N</v>
+        <v>HA10_P</v>
       </c>
       <c r="B8">
         <f>HPC_Setup_Sheet!C8</f>
@@ -3733,7 +3722,7 @@
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f>HPC_Setup_Sheet!B9</f>
-        <v>HA10_P</v>
+        <v>HA10_N</v>
       </c>
       <c r="B9">
         <f>HPC_Setup_Sheet!C9</f>
@@ -3747,7 +3736,7 @@
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f>HPC_Setup_Sheet!B10</f>
-        <v>HA10_N</v>
+        <v>HA17_P_CC</v>
       </c>
       <c r="B10">
         <f>HPC_Setup_Sheet!C10</f>
@@ -3761,7 +3750,7 @@
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f>HPC_Setup_Sheet!B11</f>
-        <v>HA17_P_CC</v>
+        <v>HA17_N_CC</v>
       </c>
       <c r="B11">
         <f>HPC_Setup_Sheet!C11</f>
@@ -3775,7 +3764,7 @@
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f>HPC_Setup_Sheet!B12</f>
-        <v>HA17_N_CC</v>
+        <v>HA21_P</v>
       </c>
       <c r="B12">
         <f>HPC_Setup_Sheet!C12</f>
@@ -3789,7 +3778,7 @@
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f>HPC_Setup_Sheet!B13</f>
-        <v>HA21_P</v>
+        <v>HA21_N</v>
       </c>
       <c r="B13">
         <f>HPC_Setup_Sheet!C13</f>
@@ -3803,7 +3792,7 @@
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f>HPC_Setup_Sheet!B14</f>
-        <v>HA21_N</v>
+        <v>HA23_P</v>
       </c>
       <c r="B14">
         <f>HPC_Setup_Sheet!C14</f>
@@ -3817,7 +3806,7 @@
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f>HPC_Setup_Sheet!B15</f>
-        <v>HA23_P</v>
+        <v>HA23_N</v>
       </c>
       <c r="B15">
         <f>HPC_Setup_Sheet!C15</f>
@@ -3831,7 +3820,7 @@
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f>HPC_Setup_Sheet!B16</f>
-        <v>HA23_N</v>
+        <v>HB00_P_CC</v>
       </c>
       <c r="B16">
         <f>HPC_Setup_Sheet!C16</f>
@@ -3845,7 +3834,7 @@
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>HPC_Setup_Sheet!B17</f>
-        <v>HB00_P_CC</v>
+        <v>HB00_N_CC</v>
       </c>
       <c r="B17">
         <f>HPC_Setup_Sheet!C17</f>
@@ -3859,7 +3848,7 @@
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>HPC_Setup_Sheet!B18</f>
-        <v>HB00_N_CC</v>
+        <v>HB06_P_CC</v>
       </c>
       <c r="B18">
         <f>HPC_Setup_Sheet!C18</f>
@@ -3873,7 +3862,7 @@
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>HPC_Setup_Sheet!B19</f>
-        <v>HB06_P_CC</v>
+        <v>HB06_N_CC</v>
       </c>
       <c r="B19">
         <f>HPC_Setup_Sheet!C19</f>
@@ -3887,7 +3876,7 @@
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>HPC_Setup_Sheet!B20</f>
-        <v>HB06_N_CC</v>
+        <v>HB10_P</v>
       </c>
       <c r="B20">
         <f>HPC_Setup_Sheet!C20</f>
@@ -3901,7 +3890,7 @@
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>HPC_Setup_Sheet!B21</f>
-        <v>HB10_P</v>
+        <v>HB10_N</v>
       </c>
       <c r="B21">
         <f>HPC_Setup_Sheet!C21</f>
@@ -3915,7 +3904,7 @@
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f>HPC_Setup_Sheet!B22</f>
-        <v>HB10_N</v>
+        <v>HB14_P</v>
       </c>
       <c r="B22">
         <f>HPC_Setup_Sheet!C22</f>
@@ -3929,7 +3918,7 @@
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f>HPC_Setup_Sheet!B23</f>
-        <v>HB14_P</v>
+        <v>HB14_N</v>
       </c>
       <c r="B23">
         <f>HPC_Setup_Sheet!C23</f>
@@ -3943,7 +3932,7 @@
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>HPC_Setup_Sheet!B24</f>
-        <v>HB14_N</v>
+        <v>HB17_P_CC</v>
       </c>
       <c r="B24">
         <f>HPC_Setup_Sheet!C24</f>
@@ -3957,7 +3946,7 @@
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f>HPC_Setup_Sheet!B25</f>
-        <v>HB17_P_CC</v>
+        <v>HB17_N_CC</v>
       </c>
       <c r="B25">
         <f>HPC_Setup_Sheet!C25</f>
@@ -3971,7 +3960,7 @@
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f>HPC_Setup_Sheet!B26</f>
-        <v>HB17_N_CC</v>
+        <v>CLK3_BIDIR_P</v>
       </c>
       <c r="B26">
         <f>HPC_Setup_Sheet!C26</f>
@@ -3985,7 +3974,7 @@
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f>HPC_Setup_Sheet!B27</f>
-        <v>CLK3_BIDIR_P</v>
+        <v>CLK3_BIDIR_N</v>
       </c>
       <c r="B27">
         <f>HPC_Setup_Sheet!C27</f>
@@ -3999,7 +3988,7 @@
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f>HPC_Setup_Sheet!B28</f>
-        <v>CLK3_BIDIR_N</v>
+        <v>HA03_P</v>
       </c>
       <c r="B28">
         <f>HPC_Setup_Sheet!C28</f>
@@ -4013,7 +4002,7 @@
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f>HPC_Setup_Sheet!B29</f>
-        <v>HA03_P</v>
+        <v>HA03_N</v>
       </c>
       <c r="B29">
         <f>HPC_Setup_Sheet!C29</f>
@@ -4027,7 +4016,7 @@
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f>HPC_Setup_Sheet!B30</f>
-        <v>HA03_N</v>
+        <v>HA07_P</v>
       </c>
       <c r="B30">
         <f>HPC_Setup_Sheet!C30</f>
@@ -4041,7 +4030,7 @@
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f>HPC_Setup_Sheet!B31</f>
-        <v>HA07_P</v>
+        <v>HA07_N</v>
       </c>
       <c r="B31">
         <f>HPC_Setup_Sheet!C31</f>
@@ -4055,7 +4044,7 @@
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f>HPC_Setup_Sheet!B32</f>
-        <v>HA07_N</v>
+        <v>HA11_P</v>
       </c>
       <c r="B32">
         <f>HPC_Setup_Sheet!C32</f>
@@ -4069,7 +4058,7 @@
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f>HPC_Setup_Sheet!B33</f>
-        <v>HA11_P</v>
+        <v>HA11_N</v>
       </c>
       <c r="B33">
         <f>HPC_Setup_Sheet!C33</f>
@@ -4083,7 +4072,7 @@
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f>HPC_Setup_Sheet!B34</f>
-        <v>HA11_N</v>
+        <v>HA14_P</v>
       </c>
       <c r="B34">
         <f>HPC_Setup_Sheet!C34</f>
@@ -4097,7 +4086,7 @@
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f>HPC_Setup_Sheet!B35</f>
-        <v>HA14_P</v>
+        <v>HA14_N</v>
       </c>
       <c r="B35">
         <f>HPC_Setup_Sheet!C35</f>
@@ -4111,7 +4100,7 @@
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f>HPC_Setup_Sheet!B36</f>
-        <v>HA14_N</v>
+        <v>HA18_P</v>
       </c>
       <c r="B36">
         <f>HPC_Setup_Sheet!C36</f>
@@ -4125,7 +4114,7 @@
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f>HPC_Setup_Sheet!B37</f>
-        <v>HA18_P</v>
+        <v>HA18_N</v>
       </c>
       <c r="B37">
         <f>HPC_Setup_Sheet!C37</f>
@@ -4139,7 +4128,7 @@
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f>HPC_Setup_Sheet!B38</f>
-        <v>HA18_N</v>
+        <v>HA22_P</v>
       </c>
       <c r="B38">
         <f>HPC_Setup_Sheet!C38</f>
@@ -4153,7 +4142,7 @@
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f>HPC_Setup_Sheet!B39</f>
-        <v>HA22_P</v>
+        <v>HA22_N</v>
       </c>
       <c r="B39">
         <f>HPC_Setup_Sheet!C39</f>
@@ -4167,7 +4156,7 @@
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f>HPC_Setup_Sheet!B40</f>
-        <v>HA22_N</v>
+        <v>HB01_P</v>
       </c>
       <c r="B40">
         <f>HPC_Setup_Sheet!C40</f>
@@ -4181,7 +4170,7 @@
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f>HPC_Setup_Sheet!B41</f>
-        <v>HB01_P</v>
+        <v>HB01_N</v>
       </c>
       <c r="B41">
         <f>HPC_Setup_Sheet!C41</f>
@@ -4195,7 +4184,7 @@
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f>HPC_Setup_Sheet!B42</f>
-        <v>HB01_N</v>
+        <v>HB07_P</v>
       </c>
       <c r="B42">
         <f>HPC_Setup_Sheet!C42</f>
@@ -4209,7 +4198,7 @@
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f>HPC_Setup_Sheet!B43</f>
-        <v>HB07_P</v>
+        <v>HB07_N</v>
       </c>
       <c r="B43">
         <f>HPC_Setup_Sheet!C43</f>
@@ -4223,7 +4212,7 @@
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f>HPC_Setup_Sheet!B44</f>
-        <v>HB07_N</v>
+        <v>HB11_P</v>
       </c>
       <c r="B44">
         <f>HPC_Setup_Sheet!C44</f>
@@ -4237,7 +4226,7 @@
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f>HPC_Setup_Sheet!B45</f>
-        <v>HB11_P</v>
+        <v>HB11_N</v>
       </c>
       <c r="B45">
         <f>HPC_Setup_Sheet!C45</f>
@@ -4251,7 +4240,7 @@
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f>HPC_Setup_Sheet!B46</f>
-        <v>HB11_N</v>
+        <v>HB15_P</v>
       </c>
       <c r="B46">
         <f>HPC_Setup_Sheet!C46</f>
@@ -4265,7 +4254,7 @@
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f>HPC_Setup_Sheet!B47</f>
-        <v>HB15_P</v>
+        <v>HB15_N</v>
       </c>
       <c r="B47">
         <f>HPC_Setup_Sheet!C47</f>
@@ -4279,7 +4268,7 @@
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f>HPC_Setup_Sheet!B48</f>
-        <v>HB15_N</v>
+        <v>HB18_P</v>
       </c>
       <c r="B48">
         <f>HPC_Setup_Sheet!C48</f>
@@ -4293,7 +4282,7 @@
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f>HPC_Setup_Sheet!B49</f>
-        <v>HB18_P</v>
+        <v>HB18_N</v>
       </c>
       <c r="B49">
         <f>HPC_Setup_Sheet!C49</f>
@@ -4307,7 +4296,7 @@
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
         <f>HPC_Setup_Sheet!B50</f>
-        <v>HB18_N</v>
+        <v>CLK0_M2C_P</v>
       </c>
       <c r="B50">
         <f>HPC_Setup_Sheet!C50</f>
@@ -4321,7 +4310,7 @@
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
         <f>HPC_Setup_Sheet!B51</f>
-        <v>CLK0_M2C_P</v>
+        <v>CLK0_M2C_N</v>
       </c>
       <c r="B51">
         <f>HPC_Setup_Sheet!C51</f>
@@ -4335,7 +4324,7 @@
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
         <f>HPC_Setup_Sheet!B52</f>
-        <v>CLK0_M2C_N</v>
+        <v>LA02_P</v>
       </c>
       <c r="B52">
         <f>HPC_Setup_Sheet!C52</f>
@@ -4349,7 +4338,7 @@
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
         <f>HPC_Setup_Sheet!B53</f>
-        <v>LA02_P</v>
+        <v>LA02_N</v>
       </c>
       <c r="B53">
         <f>HPC_Setup_Sheet!C53</f>
@@ -4363,7 +4352,7 @@
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
         <f>HPC_Setup_Sheet!B54</f>
-        <v>LA02_N</v>
+        <v>LA04_P</v>
       </c>
       <c r="B54">
         <f>HPC_Setup_Sheet!C54</f>
@@ -4377,7 +4366,7 @@
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
         <f>HPC_Setup_Sheet!B55</f>
-        <v>LA04_P</v>
+        <v>LA04_N</v>
       </c>
       <c r="B55">
         <f>HPC_Setup_Sheet!C55</f>
@@ -4391,7 +4380,7 @@
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
         <f>HPC_Setup_Sheet!B56</f>
-        <v>LA04_N</v>
+        <v>LA07_P</v>
       </c>
       <c r="B56">
         <f>HPC_Setup_Sheet!C56</f>
@@ -4405,7 +4394,7 @@
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <f>HPC_Setup_Sheet!B57</f>
-        <v>LA07_P</v>
+        <v>LA07_N</v>
       </c>
       <c r="B57">
         <f>HPC_Setup_Sheet!C57</f>
@@ -4419,7 +4408,7 @@
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
         <f>HPC_Setup_Sheet!B58</f>
-        <v>LA07_N</v>
+        <v>LA11_P</v>
       </c>
       <c r="B58">
         <f>HPC_Setup_Sheet!C58</f>
@@ -4433,7 +4422,7 @@
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="str">
         <f>HPC_Setup_Sheet!B59</f>
-        <v>LA11_P</v>
+        <v>LA11_N</v>
       </c>
       <c r="B59">
         <f>HPC_Setup_Sheet!C59</f>
@@ -4447,7 +4436,7 @@
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="str">
         <f>HPC_Setup_Sheet!B60</f>
-        <v>LA11_N</v>
+        <v>LA15_P</v>
       </c>
       <c r="B60">
         <f>HPC_Setup_Sheet!C60</f>
@@ -4461,7 +4450,7 @@
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="str">
         <f>HPC_Setup_Sheet!B61</f>
-        <v>LA15_P</v>
+        <v>LA15_N</v>
       </c>
       <c r="B61">
         <f>HPC_Setup_Sheet!C61</f>
@@ -4475,7 +4464,7 @@
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="str">
         <f>HPC_Setup_Sheet!B62</f>
-        <v>LA15_N</v>
+        <v>LA19_P</v>
       </c>
       <c r="B62">
         <f>HPC_Setup_Sheet!C62</f>
@@ -4489,7 +4478,7 @@
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="str">
         <f>HPC_Setup_Sheet!B63</f>
-        <v>LA19_P</v>
+        <v>LA19_N</v>
       </c>
       <c r="B63">
         <f>HPC_Setup_Sheet!C63</f>
@@ -4503,7 +4492,7 @@
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="str">
         <f>HPC_Setup_Sheet!B64</f>
-        <v>LA19_N</v>
+        <v>LA21_P</v>
       </c>
       <c r="B64">
         <f>HPC_Setup_Sheet!C64</f>
@@ -4517,7 +4506,7 @@
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f>HPC_Setup_Sheet!B65</f>
-        <v>LA21_P</v>
+        <v>LA21_N</v>
       </c>
       <c r="B65">
         <f>HPC_Setup_Sheet!C65</f>
@@ -4531,7 +4520,7 @@
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f>HPC_Setup_Sheet!B66</f>
-        <v>LA21_N</v>
+        <v>LA24_P</v>
       </c>
       <c r="B66">
         <f>HPC_Setup_Sheet!C66</f>
@@ -4545,7 +4534,7 @@
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f>HPC_Setup_Sheet!B67</f>
-        <v>LA24_P</v>
+        <v>LA24_N</v>
       </c>
       <c r="B67">
         <f>HPC_Setup_Sheet!C67</f>
@@ -4559,7 +4548,7 @@
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f>HPC_Setup_Sheet!B68</f>
-        <v>LA24_N</v>
+        <v>LA28_P</v>
       </c>
       <c r="B68">
         <f>HPC_Setup_Sheet!C68</f>
@@ -4573,7 +4562,7 @@
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f>HPC_Setup_Sheet!B69</f>
-        <v>LA28_P</v>
+        <v>LA28_N</v>
       </c>
       <c r="B69">
         <f>HPC_Setup_Sheet!C69</f>
@@ -4587,7 +4576,7 @@
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f>HPC_Setup_Sheet!B70</f>
-        <v>LA28_N</v>
+        <v>LA30_P</v>
       </c>
       <c r="B70">
         <f>HPC_Setup_Sheet!C70</f>
@@ -4601,7 +4590,7 @@
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f>HPC_Setup_Sheet!B71</f>
-        <v>LA30_P</v>
+        <v>LA30_N</v>
       </c>
       <c r="B71">
         <f>HPC_Setup_Sheet!C71</f>
@@ -4615,7 +4604,7 @@
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f>HPC_Setup_Sheet!B72</f>
-        <v>LA30_N</v>
+        <v>LA32_P</v>
       </c>
       <c r="B72">
         <f>HPC_Setup_Sheet!C72</f>
@@ -4629,7 +4618,7 @@
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f>HPC_Setup_Sheet!B73</f>
-        <v>LA32_P</v>
+        <v>LA32_N</v>
       </c>
       <c r="B73">
         <f>HPC_Setup_Sheet!C73</f>
@@ -4643,7 +4632,7 @@
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f>HPC_Setup_Sheet!B74</f>
-        <v>LA32_N</v>
+        <v>CLK1_M2C_P</v>
       </c>
       <c r="B74">
         <f>HPC_Setup_Sheet!C74</f>
@@ -4657,7 +4646,7 @@
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f>HPC_Setup_Sheet!B75</f>
-        <v>CLK1_M2C_P</v>
+        <v>CLK1_M2C_N</v>
       </c>
       <c r="B75">
         <f>HPC_Setup_Sheet!C75</f>
@@ -4671,7 +4660,7 @@
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f>HPC_Setup_Sheet!B76</f>
-        <v>CLK1_M2C_N</v>
+        <v>LA00_P_CC</v>
       </c>
       <c r="B76">
         <f>HPC_Setup_Sheet!C76</f>
@@ -4685,7 +4674,7 @@
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f>HPC_Setup_Sheet!B77</f>
-        <v>LA00_P_CC</v>
+        <v>LA00_N_CC</v>
       </c>
       <c r="B77">
         <f>HPC_Setup_Sheet!C77</f>
@@ -4699,7 +4688,7 @@
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f>HPC_Setup_Sheet!B78</f>
-        <v>LA00_N_CC</v>
+        <v>LA03_P</v>
       </c>
       <c r="B78">
         <f>HPC_Setup_Sheet!C78</f>
@@ -4713,7 +4702,7 @@
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f>HPC_Setup_Sheet!B79</f>
-        <v>LA03_P</v>
+        <v>LA03_N</v>
       </c>
       <c r="B79">
         <f>HPC_Setup_Sheet!C79</f>
@@ -4727,7 +4716,7 @@
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f>HPC_Setup_Sheet!B80</f>
-        <v>LA03_N</v>
+        <v>LA08_P</v>
       </c>
       <c r="B80">
         <f>HPC_Setup_Sheet!C80</f>
@@ -4741,7 +4730,7 @@
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="str">
         <f>HPC_Setup_Sheet!B81</f>
-        <v>LA08_P</v>
+        <v>LA08_N</v>
       </c>
       <c r="B81">
         <f>HPC_Setup_Sheet!C81</f>
@@ -4755,7 +4744,7 @@
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
         <f>HPC_Setup_Sheet!B82</f>
-        <v>LA08_N</v>
+        <v>LA12_P</v>
       </c>
       <c r="B82">
         <f>HPC_Setup_Sheet!C82</f>
@@ -4769,7 +4758,7 @@
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f>HPC_Setup_Sheet!B83</f>
-        <v>LA12_P</v>
+        <v>LA12_N</v>
       </c>
       <c r="B83">
         <f>HPC_Setup_Sheet!C83</f>
@@ -4783,7 +4772,7 @@
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
         <f>HPC_Setup_Sheet!B84</f>
-        <v>LA12_N</v>
+        <v>LA16_P</v>
       </c>
       <c r="B84">
         <f>HPC_Setup_Sheet!C84</f>
@@ -4797,7 +4786,7 @@
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
         <f>HPC_Setup_Sheet!B85</f>
-        <v>LA16_P</v>
+        <v>LA16_N</v>
       </c>
       <c r="B85">
         <f>HPC_Setup_Sheet!C85</f>
@@ -4811,7 +4800,7 @@
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
         <f>HPC_Setup_Sheet!B86</f>
-        <v>LA16_N</v>
+        <v>LA20_P</v>
       </c>
       <c r="B86">
         <f>HPC_Setup_Sheet!C86</f>
@@ -4825,7 +4814,7 @@
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="str">
         <f>HPC_Setup_Sheet!B87</f>
-        <v>LA20_P</v>
+        <v>LA20_N</v>
       </c>
       <c r="B87">
         <f>HPC_Setup_Sheet!C87</f>
@@ -4839,7 +4828,7 @@
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="str">
         <f>HPC_Setup_Sheet!B88</f>
-        <v>LA20_N</v>
+        <v>LA22_P</v>
       </c>
       <c r="B88">
         <f>HPC_Setup_Sheet!C88</f>
@@ -4853,7 +4842,7 @@
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="str">
         <f>HPC_Setup_Sheet!B89</f>
-        <v>LA22_P</v>
+        <v>LA22_N</v>
       </c>
       <c r="B89">
         <f>HPC_Setup_Sheet!C89</f>
@@ -4867,7 +4856,7 @@
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <f>HPC_Setup_Sheet!B90</f>
-        <v>LA22_N</v>
+        <v>LA25_P</v>
       </c>
       <c r="B90">
         <f>HPC_Setup_Sheet!C90</f>
@@ -4881,7 +4870,7 @@
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
         <f>HPC_Setup_Sheet!B91</f>
-        <v>LA25_P</v>
+        <v>LA25_N</v>
       </c>
       <c r="B91">
         <f>HPC_Setup_Sheet!C91</f>
@@ -4895,7 +4884,7 @@
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
         <f>HPC_Setup_Sheet!B92</f>
-        <v>LA25_N</v>
+        <v>LA29_P</v>
       </c>
       <c r="B92">
         <f>HPC_Setup_Sheet!C92</f>
@@ -4909,7 +4898,7 @@
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
         <f>HPC_Setup_Sheet!B93</f>
-        <v>LA29_P</v>
+        <v>LA29_N</v>
       </c>
       <c r="B93">
         <f>HPC_Setup_Sheet!C93</f>
@@ -4923,7 +4912,7 @@
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="str">
         <f>HPC_Setup_Sheet!B94</f>
-        <v>LA29_N</v>
+        <v>LA31_P</v>
       </c>
       <c r="B94">
         <f>HPC_Setup_Sheet!C94</f>
@@ -4937,7 +4926,7 @@
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="str">
         <f>HPC_Setup_Sheet!B95</f>
-        <v>LA31_P</v>
+        <v>LA31_N</v>
       </c>
       <c r="B95">
         <f>HPC_Setup_Sheet!C95</f>
@@ -4951,7 +4940,7 @@
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="str">
         <f>HPC_Setup_Sheet!B96</f>
-        <v>LA31_N</v>
+        <v>LA33_P</v>
       </c>
       <c r="B96">
         <f>HPC_Setup_Sheet!C96</f>
@@ -4965,7 +4954,7 @@
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="str">
         <f>HPC_Setup_Sheet!B97</f>
-        <v>LA33_P</v>
+        <v>LA33_N</v>
       </c>
       <c r="B97">
         <f>HPC_Setup_Sheet!C97</f>
@@ -4979,7 +4968,7 @@
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="str">
         <f>HPC_Setup_Sheet!B98</f>
-        <v>LA33_N</v>
+        <v>HA00_P_CC</v>
       </c>
       <c r="B98">
         <f>HPC_Setup_Sheet!C98</f>
@@ -4993,7 +4982,7 @@
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="str">
         <f>HPC_Setup_Sheet!B99</f>
-        <v>HA00_P_CC</v>
+        <v>HA00_N_CC</v>
       </c>
       <c r="B99">
         <f>HPC_Setup_Sheet!C99</f>
@@ -5007,7 +4996,7 @@
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="str">
         <f>HPC_Setup_Sheet!B100</f>
-        <v>HA00_N_CC</v>
+        <v>HA04_P</v>
       </c>
       <c r="B100">
         <f>HPC_Setup_Sheet!C100</f>
@@ -5021,7 +5010,7 @@
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="str">
         <f>HPC_Setup_Sheet!B101</f>
-        <v>HA04_P</v>
+        <v>HA04_N</v>
       </c>
       <c r="B101">
         <f>HPC_Setup_Sheet!C101</f>
@@ -5035,7 +5024,7 @@
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="str">
         <f>HPC_Setup_Sheet!B102</f>
-        <v>HA04_N</v>
+        <v>HA08_P</v>
       </c>
       <c r="B102">
         <f>HPC_Setup_Sheet!C102</f>
@@ -5049,7 +5038,7 @@
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="str">
         <f>HPC_Setup_Sheet!B103</f>
-        <v>HA08_P</v>
+        <v>HA08_N</v>
       </c>
       <c r="B103">
         <f>HPC_Setup_Sheet!C103</f>
@@ -5063,7 +5052,7 @@
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="str">
         <f>HPC_Setup_Sheet!B104</f>
-        <v>HA08_N</v>
+        <v>HA12_P</v>
       </c>
       <c r="B104">
         <f>HPC_Setup_Sheet!C104</f>
@@ -5077,7 +5066,7 @@
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="str">
         <f>HPC_Setup_Sheet!B105</f>
-        <v>HA12_P</v>
+        <v>HA12_N</v>
       </c>
       <c r="B105">
         <f>HPC_Setup_Sheet!C105</f>
@@ -5091,7 +5080,7 @@
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="str">
         <f>HPC_Setup_Sheet!B106</f>
-        <v>HA12_N</v>
+        <v>HA15_P</v>
       </c>
       <c r="B106">
         <f>HPC_Setup_Sheet!C106</f>
@@ -5105,7 +5094,7 @@
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="str">
         <f>HPC_Setup_Sheet!B107</f>
-        <v>HA15_P</v>
+        <v>HA15_N</v>
       </c>
       <c r="B107">
         <f>HPC_Setup_Sheet!C107</f>
@@ -5119,7 +5108,7 @@
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="str">
         <f>HPC_Setup_Sheet!B108</f>
-        <v>HA15_N</v>
+        <v>HA19_P</v>
       </c>
       <c r="B108">
         <f>HPC_Setup_Sheet!C108</f>
@@ -5133,7 +5122,7 @@
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="str">
         <f>HPC_Setup_Sheet!B109</f>
-        <v>HA19_P</v>
+        <v>HA19_N</v>
       </c>
       <c r="B109">
         <f>HPC_Setup_Sheet!C109</f>
@@ -5147,7 +5136,7 @@
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="str">
         <f>HPC_Setup_Sheet!B110</f>
-        <v>HA19_N</v>
+        <v>HB02_P</v>
       </c>
       <c r="B110">
         <f>HPC_Setup_Sheet!C110</f>
@@ -5161,7 +5150,7 @@
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="str">
         <f>HPC_Setup_Sheet!B111</f>
-        <v>HB02_P</v>
+        <v>HB02_N</v>
       </c>
       <c r="B111">
         <f>HPC_Setup_Sheet!C111</f>
@@ -5175,7 +5164,7 @@
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="str">
         <f>HPC_Setup_Sheet!B112</f>
-        <v>HB02_N</v>
+        <v>HB04_P</v>
       </c>
       <c r="B112">
         <f>HPC_Setup_Sheet!C112</f>
@@ -5189,7 +5178,7 @@
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="str">
         <f>HPC_Setup_Sheet!B113</f>
-        <v>HB04_P</v>
+        <v>HB04_N</v>
       </c>
       <c r="B113">
         <f>HPC_Setup_Sheet!C113</f>
@@ -5203,7 +5192,7 @@
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="str">
         <f>HPC_Setup_Sheet!B114</f>
-        <v>HB04_N</v>
+        <v>HB08_P</v>
       </c>
       <c r="B114">
         <f>HPC_Setup_Sheet!C114</f>
@@ -5217,7 +5206,7 @@
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="str">
         <f>HPC_Setup_Sheet!B115</f>
-        <v>HB08_P</v>
+        <v>HB08_N</v>
       </c>
       <c r="B115">
         <f>HPC_Setup_Sheet!C115</f>
@@ -5231,7 +5220,7 @@
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="str">
         <f>HPC_Setup_Sheet!B116</f>
-        <v>HB08_N</v>
+        <v>HB12_P</v>
       </c>
       <c r="B116">
         <f>HPC_Setup_Sheet!C116</f>
@@ -5245,7 +5234,7 @@
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="str">
         <f>HPC_Setup_Sheet!B117</f>
-        <v>HB12_P</v>
+        <v>HB12_N</v>
       </c>
       <c r="B117">
         <f>HPC_Setup_Sheet!C117</f>
@@ -5259,7 +5248,7 @@
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="str">
         <f>HPC_Setup_Sheet!B118</f>
-        <v>HB12_N</v>
+        <v>HB16_P</v>
       </c>
       <c r="B118">
         <f>HPC_Setup_Sheet!C118</f>
@@ -5273,7 +5262,7 @@
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="str">
         <f>HPC_Setup_Sheet!B119</f>
-        <v>HB16_P</v>
+        <v>HB16_N</v>
       </c>
       <c r="B119">
         <f>HPC_Setup_Sheet!C119</f>
@@ -5287,7 +5276,7 @@
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="str">
         <f>HPC_Setup_Sheet!B120</f>
-        <v>HB16_N</v>
+        <v>HB20_P</v>
       </c>
       <c r="B120">
         <f>HPC_Setup_Sheet!C120</f>
@@ -5301,7 +5290,7 @@
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="str">
         <f>HPC_Setup_Sheet!B121</f>
-        <v>HB20_P</v>
+        <v>HB20_N</v>
       </c>
       <c r="B121">
         <f>HPC_Setup_Sheet!C121</f>
@@ -5315,7 +5304,7 @@
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="str">
         <f>HPC_Setup_Sheet!B122</f>
-        <v>HB20_N</v>
+        <v>HA01_P_CC</v>
       </c>
       <c r="B122">
         <f>HPC_Setup_Sheet!C122</f>
@@ -5329,7 +5318,7 @@
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="str">
         <f>HPC_Setup_Sheet!B123</f>
-        <v>HA01_P_CC</v>
+        <v>HA01_N_CC</v>
       </c>
       <c r="B123">
         <f>HPC_Setup_Sheet!C123</f>
@@ -5343,7 +5332,7 @@
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="str">
         <f>HPC_Setup_Sheet!B124</f>
-        <v>HA01_N_CC</v>
+        <v>HA05_P</v>
       </c>
       <c r="B124">
         <f>HPC_Setup_Sheet!C124</f>
@@ -5357,7 +5346,7 @@
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="str">
         <f>HPC_Setup_Sheet!B125</f>
-        <v>HA05_P</v>
+        <v>HA05_N</v>
       </c>
       <c r="B125">
         <f>HPC_Setup_Sheet!C125</f>
@@ -5371,7 +5360,7 @@
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="str">
         <f>HPC_Setup_Sheet!B126</f>
-        <v>HA05_N</v>
+        <v>HA09_P</v>
       </c>
       <c r="B126">
         <f>HPC_Setup_Sheet!C126</f>
@@ -5385,7 +5374,7 @@
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="str">
         <f>HPC_Setup_Sheet!B127</f>
-        <v>HA09_P</v>
+        <v>HA09_N</v>
       </c>
       <c r="B127">
         <f>HPC_Setup_Sheet!C127</f>
@@ -5399,7 +5388,7 @@
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="str">
         <f>HPC_Setup_Sheet!B128</f>
-        <v>HA09_N</v>
+        <v>HA13_P</v>
       </c>
       <c r="B128">
         <f>HPC_Setup_Sheet!C128</f>
@@ -5413,7 +5402,7 @@
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="str">
         <f>HPC_Setup_Sheet!B129</f>
-        <v>HA13_P</v>
+        <v>HA13_N</v>
       </c>
       <c r="B129">
         <f>HPC_Setup_Sheet!C129</f>
@@ -5427,7 +5416,7 @@
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="str">
         <f>HPC_Setup_Sheet!B130</f>
-        <v>HA13_N</v>
+        <v>HA16_P</v>
       </c>
       <c r="B130">
         <f>HPC_Setup_Sheet!C130</f>
@@ -5441,7 +5430,7 @@
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="str">
         <f>HPC_Setup_Sheet!B131</f>
-        <v>HA16_P</v>
+        <v>HA16_N</v>
       </c>
       <c r="B131">
         <f>HPC_Setup_Sheet!C131</f>
@@ -5455,7 +5444,7 @@
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="str">
         <f>HPC_Setup_Sheet!B132</f>
-        <v>HA16_N</v>
+        <v>HA20_P</v>
       </c>
       <c r="B132">
         <f>HPC_Setup_Sheet!C132</f>
@@ -5469,7 +5458,7 @@
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="str">
         <f>HPC_Setup_Sheet!B133</f>
-        <v>HA20_P</v>
+        <v>HA20_N</v>
       </c>
       <c r="B133">
         <f>HPC_Setup_Sheet!C133</f>
@@ -5483,7 +5472,7 @@
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="str">
         <f>HPC_Setup_Sheet!B134</f>
-        <v>HA20_N</v>
+        <v>HB03_P</v>
       </c>
       <c r="B134">
         <f>HPC_Setup_Sheet!C134</f>
@@ -5497,7 +5486,7 @@
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="str">
         <f>HPC_Setup_Sheet!B135</f>
-        <v>HB03_P</v>
+        <v>HB03_N</v>
       </c>
       <c r="B135">
         <f>HPC_Setup_Sheet!C135</f>
@@ -5511,7 +5500,7 @@
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="str">
         <f>HPC_Setup_Sheet!B136</f>
-        <v>HB03_N</v>
+        <v>HB05_P</v>
       </c>
       <c r="B136">
         <f>HPC_Setup_Sheet!C136</f>
@@ -5525,7 +5514,7 @@
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="str">
         <f>HPC_Setup_Sheet!B137</f>
-        <v>HB05_P</v>
+        <v>HB05_N</v>
       </c>
       <c r="B137">
         <f>HPC_Setup_Sheet!C137</f>
@@ -5539,7 +5528,7 @@
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="str">
         <f>HPC_Setup_Sheet!B138</f>
-        <v>HB05_N</v>
+        <v>HB09_P</v>
       </c>
       <c r="B138">
         <f>HPC_Setup_Sheet!C138</f>
@@ -5553,7 +5542,7 @@
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="str">
         <f>HPC_Setup_Sheet!B139</f>
-        <v>HB09_P</v>
+        <v>HB09_N</v>
       </c>
       <c r="B139">
         <f>HPC_Setup_Sheet!C139</f>
@@ -5567,7 +5556,7 @@
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="str">
         <f>HPC_Setup_Sheet!B140</f>
-        <v>HB09_N</v>
+        <v>HB13_P</v>
       </c>
       <c r="B140">
         <f>HPC_Setup_Sheet!C140</f>
@@ -5581,7 +5570,7 @@
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="str">
         <f>HPC_Setup_Sheet!B141</f>
-        <v>HB13_P</v>
+        <v>HB13_N</v>
       </c>
       <c r="B141">
         <f>HPC_Setup_Sheet!C141</f>
@@ -5595,7 +5584,7 @@
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="str">
         <f>HPC_Setup_Sheet!B142</f>
-        <v>HB13_N</v>
+        <v>HB19_P</v>
       </c>
       <c r="B142">
         <f>HPC_Setup_Sheet!C142</f>
@@ -5609,7 +5598,7 @@
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="str">
         <f>HPC_Setup_Sheet!B143</f>
-        <v>HB19_P</v>
+        <v>HB19_N</v>
       </c>
       <c r="B143">
         <f>HPC_Setup_Sheet!C143</f>
@@ -5623,7 +5612,7 @@
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="str">
         <f>HPC_Setup_Sheet!B144</f>
-        <v>HB19_N</v>
+        <v>HB21_P</v>
       </c>
       <c r="B144">
         <f>HPC_Setup_Sheet!C144</f>
@@ -5637,7 +5626,7 @@
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="str">
         <f>HPC_Setup_Sheet!B145</f>
-        <v>HB21_P</v>
+        <v>HB21_N</v>
       </c>
       <c r="B145">
         <f>HPC_Setup_Sheet!C145</f>
@@ -5651,7 +5640,7 @@
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="str">
         <f>HPC_Setup_Sheet!B146</f>
-        <v>HB21_N</v>
+        <v>GBTCLK0_M2C_P</v>
       </c>
       <c r="B146">
         <f>HPC_Setup_Sheet!C146</f>
@@ -5665,7 +5654,7 @@
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="str">
         <f>HPC_Setup_Sheet!B147</f>
-        <v>GBTCLK0_M2C_P</v>
+        <v>GBTCLK0_M2C_N</v>
       </c>
       <c r="B147">
         <f>HPC_Setup_Sheet!C147</f>
@@ -5679,7 +5668,7 @@
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="str">
         <f>HPC_Setup_Sheet!B148</f>
-        <v>GBTCLK0_M2C_N</v>
+        <v>LA01_P_CC</v>
       </c>
       <c r="B148">
         <f>HPC_Setup_Sheet!C148</f>
@@ -5693,7 +5682,7 @@
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="str">
         <f>HPC_Setup_Sheet!B149</f>
-        <v>LA01_P_CC</v>
+        <v>LA01_N_CC</v>
       </c>
       <c r="B149">
         <f>HPC_Setup_Sheet!C149</f>
@@ -5707,7 +5696,7 @@
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="str">
         <f>HPC_Setup_Sheet!B150</f>
-        <v>LA01_N_CC</v>
+        <v>LA05_P</v>
       </c>
       <c r="B150">
         <f>HPC_Setup_Sheet!C150</f>
@@ -5721,7 +5710,7 @@
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="str">
         <f>HPC_Setup_Sheet!B151</f>
-        <v>LA05_P</v>
+        <v>LA05_N</v>
       </c>
       <c r="B151">
         <f>HPC_Setup_Sheet!C151</f>
@@ -5735,7 +5724,7 @@
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="str">
         <f>HPC_Setup_Sheet!B152</f>
-        <v>LA05_N</v>
+        <v>LA09_P</v>
       </c>
       <c r="B152">
         <f>HPC_Setup_Sheet!C152</f>
@@ -5749,7 +5738,7 @@
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="str">
         <f>HPC_Setup_Sheet!B153</f>
-        <v>LA09_P</v>
+        <v>LA09_N</v>
       </c>
       <c r="B153">
         <f>HPC_Setup_Sheet!C153</f>
@@ -5763,7 +5752,7 @@
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="str">
         <f>HPC_Setup_Sheet!B154</f>
-        <v>LA09_N</v>
+        <v>LA13_P</v>
       </c>
       <c r="B154">
         <f>HPC_Setup_Sheet!C154</f>
@@ -5777,7 +5766,7 @@
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="str">
         <f>HPC_Setup_Sheet!B155</f>
-        <v>LA13_P</v>
+        <v>LA13_N</v>
       </c>
       <c r="B155">
         <f>HPC_Setup_Sheet!C155</f>
@@ -5791,7 +5780,7 @@
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="str">
         <f>HPC_Setup_Sheet!B156</f>
-        <v>LA13_N</v>
+        <v>LA17_P_CC</v>
       </c>
       <c r="B156">
         <f>HPC_Setup_Sheet!C156</f>
@@ -5805,7 +5794,7 @@
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="str">
         <f>HPC_Setup_Sheet!B157</f>
-        <v>LA17_P_CC</v>
+        <v>LA17_N_CC</v>
       </c>
       <c r="B157">
         <f>HPC_Setup_Sheet!C157</f>
@@ -5819,7 +5808,7 @@
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="str">
         <f>HPC_Setup_Sheet!B158</f>
-        <v>LA17_N_CC</v>
+        <v>LA23_P</v>
       </c>
       <c r="B158">
         <f>HPC_Setup_Sheet!C158</f>
@@ -5833,7 +5822,7 @@
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="str">
         <f>HPC_Setup_Sheet!B159</f>
-        <v>LA23_P</v>
+        <v>LA23_N</v>
       </c>
       <c r="B159">
         <f>HPC_Setup_Sheet!C159</f>
@@ -5847,7 +5836,7 @@
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="str">
         <f>HPC_Setup_Sheet!B160</f>
-        <v>LA23_N</v>
+        <v>LA26_P</v>
       </c>
       <c r="B160">
         <f>HPC_Setup_Sheet!C160</f>
@@ -5861,7 +5850,7 @@
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="str">
         <f>HPC_Setup_Sheet!B161</f>
-        <v>LA26_P</v>
+        <v>LA26_N</v>
       </c>
       <c r="B161">
         <f>HPC_Setup_Sheet!C161</f>
@@ -5875,7 +5864,7 @@
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="str">
         <f>HPC_Setup_Sheet!B162</f>
-        <v>LA26_N</v>
+        <v>DP0_C2M_P</v>
       </c>
       <c r="B162">
         <f>HPC_Setup_Sheet!C162</f>
@@ -5889,7 +5878,7 @@
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="str">
         <f>HPC_Setup_Sheet!B163</f>
-        <v>DP0_C2M_P</v>
+        <v>DP0_C2M_N</v>
       </c>
       <c r="B163">
         <f>HPC_Setup_Sheet!C163</f>
@@ -5903,7 +5892,7 @@
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="str">
         <f>HPC_Setup_Sheet!B164</f>
-        <v>DP0_C2M_N</v>
+        <v>DP0_M2C_P</v>
       </c>
       <c r="B164">
         <f>HPC_Setup_Sheet!C164</f>
@@ -5917,7 +5906,7 @@
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="str">
         <f>HPC_Setup_Sheet!B165</f>
-        <v>DP0_M2C_P</v>
+        <v>DP0_M2C_N</v>
       </c>
       <c r="B165">
         <f>HPC_Setup_Sheet!C165</f>
@@ -5931,7 +5920,7 @@
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="str">
         <f>HPC_Setup_Sheet!B166</f>
-        <v>DP0_M2C_N</v>
+        <v>LA06_P</v>
       </c>
       <c r="B166">
         <f>HPC_Setup_Sheet!C166</f>
@@ -5945,7 +5934,7 @@
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="str">
         <f>HPC_Setup_Sheet!B167</f>
-        <v>LA06_P</v>
+        <v>LA06_N</v>
       </c>
       <c r="B167">
         <f>HPC_Setup_Sheet!C167</f>
@@ -5959,7 +5948,7 @@
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="str">
         <f>HPC_Setup_Sheet!B168</f>
-        <v>LA06_N</v>
+        <v>LA10_P</v>
       </c>
       <c r="B168">
         <f>HPC_Setup_Sheet!C168</f>
@@ -5973,7 +5962,7 @@
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="str">
         <f>HPC_Setup_Sheet!B169</f>
-        <v>LA10_P</v>
+        <v>LA10_N</v>
       </c>
       <c r="B169">
         <f>HPC_Setup_Sheet!C169</f>
@@ -5987,7 +5976,7 @@
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="str">
         <f>HPC_Setup_Sheet!B170</f>
-        <v>LA10_N</v>
+        <v>LA14_P</v>
       </c>
       <c r="B170">
         <f>HPC_Setup_Sheet!C170</f>
@@ -6001,7 +5990,7 @@
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="str">
         <f>HPC_Setup_Sheet!B171</f>
-        <v>LA14_P</v>
+        <v>LA14_N</v>
       </c>
       <c r="B171">
         <f>HPC_Setup_Sheet!C171</f>
@@ -6015,7 +6004,7 @@
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="str">
         <f>HPC_Setup_Sheet!B172</f>
-        <v>LA14_N</v>
+        <v>LA18_P_CC</v>
       </c>
       <c r="B172">
         <f>HPC_Setup_Sheet!C172</f>
@@ -6029,7 +6018,7 @@
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="str">
         <f>HPC_Setup_Sheet!B173</f>
-        <v>LA18_P_CC</v>
+        <v>LA18_N_CC</v>
       </c>
       <c r="B173">
         <f>HPC_Setup_Sheet!C173</f>
@@ -6043,7 +6032,7 @@
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="str">
         <f>HPC_Setup_Sheet!B174</f>
-        <v>LA18_N_CC</v>
+        <v>LA27_P</v>
       </c>
       <c r="B174">
         <f>HPC_Setup_Sheet!C174</f>
@@ -6057,7 +6046,7 @@
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="str">
         <f>HPC_Setup_Sheet!B175</f>
-        <v>LA27_P</v>
+        <v>LA27_N</v>
       </c>
       <c r="B175">
         <f>HPC_Setup_Sheet!C175</f>
@@ -6071,7 +6060,7 @@
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="str">
         <f>HPC_Setup_Sheet!B176</f>
-        <v>LA27_N</v>
+        <v>CLK_DIR</v>
       </c>
       <c r="B176">
         <f>HPC_Setup_Sheet!C176</f>
@@ -6085,7 +6074,7 @@
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="str">
         <f>HPC_Setup_Sheet!B177</f>
-        <v>CLK_DIR</v>
+        <v>DP9_M2C_P</v>
       </c>
       <c r="B177">
         <f>HPC_Setup_Sheet!C177</f>
@@ -6099,7 +6088,7 @@
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="str">
         <f>HPC_Setup_Sheet!B178</f>
-        <v>DP9_M2C_P</v>
+        <v>DP9_M2C_N</v>
       </c>
       <c r="B178">
         <f>HPC_Setup_Sheet!C178</f>
@@ -6113,7 +6102,7 @@
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="str">
         <f>HPC_Setup_Sheet!B179</f>
-        <v>DP9_M2C_N</v>
+        <v>DP8_M2C_P</v>
       </c>
       <c r="B179">
         <f>HPC_Setup_Sheet!C179</f>
@@ -6127,7 +6116,7 @@
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="str">
         <f>HPC_Setup_Sheet!B180</f>
-        <v>DP8_M2C_P</v>
+        <v>DP8_M2C_N</v>
       </c>
       <c r="B180">
         <f>HPC_Setup_Sheet!C180</f>
@@ -6141,7 +6130,7 @@
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="str">
         <f>HPC_Setup_Sheet!B181</f>
-        <v>DP8_M2C_N</v>
+        <v>DP7_M2C_P</v>
       </c>
       <c r="B181">
         <f>HPC_Setup_Sheet!C181</f>
@@ -6155,7 +6144,7 @@
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="str">
         <f>HPC_Setup_Sheet!B182</f>
-        <v>DP7_M2C_P</v>
+        <v>DP7_M2C_N</v>
       </c>
       <c r="B182">
         <f>HPC_Setup_Sheet!C182</f>
@@ -6169,7 +6158,7 @@
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="str">
         <f>HPC_Setup_Sheet!B183</f>
-        <v>DP7_M2C_N</v>
+        <v>DP6_M2C_P</v>
       </c>
       <c r="B183">
         <f>HPC_Setup_Sheet!C183</f>
@@ -6183,7 +6172,7 @@
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="str">
         <f>HPC_Setup_Sheet!B184</f>
-        <v>DP6_M2C_P</v>
+        <v>DP6_M2C_N</v>
       </c>
       <c r="B184">
         <f>HPC_Setup_Sheet!C184</f>
@@ -6197,7 +6186,7 @@
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="str">
         <f>HPC_Setup_Sheet!B185</f>
-        <v>DP6_M2C_N</v>
+        <v>GBTCLK1_M2C_P</v>
       </c>
       <c r="B185">
         <f>HPC_Setup_Sheet!C185</f>
@@ -6211,7 +6200,7 @@
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="str">
         <f>HPC_Setup_Sheet!B186</f>
-        <v>GBTCLK1_M2C_P</v>
+        <v>GBTCLK1_M2C_N</v>
       </c>
       <c r="B186">
         <f>HPC_Setup_Sheet!C186</f>
@@ -6225,7 +6214,7 @@
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="str">
         <f>HPC_Setup_Sheet!B187</f>
-        <v>GBTCLK1_M2C_N</v>
+        <v>DP9_C2M_P</v>
       </c>
       <c r="B187">
         <f>HPC_Setup_Sheet!C187</f>
@@ -6239,7 +6228,7 @@
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="str">
         <f>HPC_Setup_Sheet!B188</f>
-        <v>DP9_C2M_P</v>
+        <v>DP9_C2M_N</v>
       </c>
       <c r="B188">
         <f>HPC_Setup_Sheet!C188</f>
@@ -6253,7 +6242,7 @@
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="str">
         <f>HPC_Setup_Sheet!B189</f>
-        <v>DP9_C2M_N</v>
+        <v>DP8_C2M_P</v>
       </c>
       <c r="B189">
         <f>HPC_Setup_Sheet!C189</f>
@@ -6267,7 +6256,7 @@
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="str">
         <f>HPC_Setup_Sheet!B190</f>
-        <v>DP8_C2M_P</v>
+        <v>DP8_C2M_N</v>
       </c>
       <c r="B190">
         <f>HPC_Setup_Sheet!C190</f>
@@ -6281,7 +6270,7 @@
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="str">
         <f>HPC_Setup_Sheet!B191</f>
-        <v>DP8_C2M_N</v>
+        <v>DP7_C2M_P</v>
       </c>
       <c r="B191">
         <f>HPC_Setup_Sheet!C191</f>
@@ -6295,7 +6284,7 @@
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="str">
         <f>HPC_Setup_Sheet!B192</f>
-        <v>DP7_C2M_P</v>
+        <v>DP7_C2M_N</v>
       </c>
       <c r="B192">
         <f>HPC_Setup_Sheet!C192</f>
@@ -6309,7 +6298,7 @@
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="str">
         <f>HPC_Setup_Sheet!B193</f>
-        <v>DP7_C2M_N</v>
+        <v>DP6_C2M_P</v>
       </c>
       <c r="B193">
         <f>HPC_Setup_Sheet!C193</f>
@@ -6323,7 +6312,7 @@
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="str">
         <f>HPC_Setup_Sheet!B194</f>
-        <v>DP6_C2M_P</v>
+        <v>DP6_C2M_N</v>
       </c>
       <c r="B194">
         <f>HPC_Setup_Sheet!C194</f>
@@ -6337,7 +6326,7 @@
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="str">
         <f>HPC_Setup_Sheet!B195</f>
-        <v>DP6_C2M_N</v>
+        <v>DP1_M2C_P</v>
       </c>
       <c r="B195">
         <f>HPC_Setup_Sheet!C195</f>
@@ -6351,7 +6340,7 @@
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="str">
         <f>HPC_Setup_Sheet!B196</f>
-        <v>DP1_M2C_P</v>
+        <v>DP1_M2C_N</v>
       </c>
       <c r="B196">
         <f>HPC_Setup_Sheet!C196</f>
@@ -6365,7 +6354,7 @@
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="str">
         <f>HPC_Setup_Sheet!B197</f>
-        <v>DP1_M2C_N</v>
+        <v>DP2_M2C_P</v>
       </c>
       <c r="B197">
         <f>HPC_Setup_Sheet!C197</f>
@@ -6379,7 +6368,7 @@
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="str">
         <f>HPC_Setup_Sheet!B198</f>
-        <v>DP2_M2C_P</v>
+        <v>DP2_M2C_N</v>
       </c>
       <c r="B198">
         <f>HPC_Setup_Sheet!C198</f>
@@ -6393,7 +6382,7 @@
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="str">
         <f>HPC_Setup_Sheet!B199</f>
-        <v>DP2_M2C_N</v>
+        <v>DP3_M2C_P</v>
       </c>
       <c r="B199">
         <f>HPC_Setup_Sheet!C199</f>
@@ -6407,7 +6396,7 @@
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="str">
         <f>HPC_Setup_Sheet!B200</f>
-        <v>DP3_M2C_P</v>
+        <v>DP3_M2C_N</v>
       </c>
       <c r="B200">
         <f>HPC_Setup_Sheet!C200</f>
@@ -6421,7 +6410,7 @@
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="str">
         <f>HPC_Setup_Sheet!B201</f>
-        <v>DP3_M2C_N</v>
+        <v>DP4_M2C_P</v>
       </c>
       <c r="B201">
         <f>HPC_Setup_Sheet!C201</f>
@@ -6435,7 +6424,7 @@
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="str">
         <f>HPC_Setup_Sheet!B202</f>
-        <v>DP4_M2C_P</v>
+        <v>DP4_M2C_N</v>
       </c>
       <c r="B202">
         <f>HPC_Setup_Sheet!C202</f>
@@ -6449,7 +6438,7 @@
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="str">
         <f>HPC_Setup_Sheet!B203</f>
-        <v>DP4_M2C_N</v>
+        <v>DP5_M2C_P</v>
       </c>
       <c r="B203">
         <f>HPC_Setup_Sheet!C203</f>
@@ -6463,7 +6452,7 @@
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="str">
         <f>HPC_Setup_Sheet!B204</f>
-        <v>DP5_M2C_P</v>
+        <v>DP5_M2C_N</v>
       </c>
       <c r="B204">
         <f>HPC_Setup_Sheet!C204</f>
@@ -6477,7 +6466,7 @@
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="str">
         <f>HPC_Setup_Sheet!B205</f>
-        <v>DP5_M2C_N</v>
+        <v>DP1_C2M_P</v>
       </c>
       <c r="B205">
         <f>HPC_Setup_Sheet!C205</f>
@@ -6491,7 +6480,7 @@
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="str">
         <f>HPC_Setup_Sheet!B206</f>
-        <v>DP1_C2M_P</v>
+        <v>DP1_C2M_N</v>
       </c>
       <c r="B206">
         <f>HPC_Setup_Sheet!C206</f>
@@ -6505,7 +6494,7 @@
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="str">
         <f>HPC_Setup_Sheet!B207</f>
-        <v>DP1_C2M_N</v>
+        <v>DP2_C2M_P</v>
       </c>
       <c r="B207">
         <f>HPC_Setup_Sheet!C207</f>
@@ -6519,7 +6508,7 @@
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="str">
         <f>HPC_Setup_Sheet!B208</f>
-        <v>DP2_C2M_P</v>
+        <v>DP2_C2M_N</v>
       </c>
       <c r="B208">
         <f>HPC_Setup_Sheet!C208</f>
@@ -6533,7 +6522,7 @@
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="str">
         <f>HPC_Setup_Sheet!B209</f>
-        <v>DP2_C2M_N</v>
+        <v>DP3_C2M_P</v>
       </c>
       <c r="B209">
         <f>HPC_Setup_Sheet!C209</f>
@@ -6547,7 +6536,7 @@
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="str">
         <f>HPC_Setup_Sheet!B210</f>
-        <v>DP3_C2M_P</v>
+        <v>DP3_C2M_N</v>
       </c>
       <c r="B210">
         <f>HPC_Setup_Sheet!C210</f>
@@ -6561,7 +6550,7 @@
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="str">
         <f>HPC_Setup_Sheet!B211</f>
-        <v>DP3_C2M_N</v>
+        <v>DP4_C2M_P</v>
       </c>
       <c r="B211">
         <f>HPC_Setup_Sheet!C211</f>
@@ -6575,7 +6564,7 @@
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="str">
         <f>HPC_Setup_Sheet!B212</f>
-        <v>DP4_C2M_P</v>
+        <v>DP4_C2M_N</v>
       </c>
       <c r="B212">
         <f>HPC_Setup_Sheet!C212</f>
@@ -6589,7 +6578,7 @@
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="str">
         <f>HPC_Setup_Sheet!B213</f>
-        <v>DP4_C2M_N</v>
+        <v>DP5_C2M_P</v>
       </c>
       <c r="B213">
         <f>HPC_Setup_Sheet!C213</f>
@@ -6603,7 +6592,7 @@
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="str">
         <f>HPC_Setup_Sheet!B214</f>
-        <v>DP5_C2M_P</v>
+        <v>DP5_C2M_N</v>
       </c>
       <c r="B214">
         <f>HPC_Setup_Sheet!C214</f>
@@ -6611,20 +6600,6 @@
       </c>
       <c r="C214" t="str">
         <f>HPC_Setup_Sheet!D214</f>
-        <v>Input</v>
-      </c>
-    </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A215" t="str">
-        <f>HPC_Setup_Sheet!B215</f>
-        <v>DP5_C2M_N</v>
-      </c>
-      <c r="B215">
-        <f>HPC_Setup_Sheet!C215</f>
-        <v>0</v>
-      </c>
-      <c r="C215" t="str">
-        <f>HPC_Setup_Sheet!D215</f>
         <v>Input</v>
       </c>
     </row>

</xml_diff>